<commit_message>
made changes in Data_Provider.java, AddambulanceAction.java, LoginAction.java, Driver.java, AddambulancePage.java, TestNGRunner.java, AddambulanceStepDefinition.java, TestData.xlsx
</commit_message>
<xml_diff>
--- a/SmartHospitalTesting/src/test/resources/test_datas/TestData.xlsx
+++ b/SmartHospitalTesting/src/test/resources/test_datas/TestData.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dhars\Documents\SmartHospitalTestingProject\SmartHospitalTesting\src\test\resources\test_datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1991792F-0C6B-4D4C-8C71-1E0B517C7986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2B5C183-F1BD-401C-A1B9-CD6936E2A11D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{EFB5B7BA-D904-4328-9088-4D5919CB03C0}"/>
+    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="8880" xr2:uid="{EFB5B7BA-D904-4328-9088-4D5919CB03C0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>patient</t>
   </si>
@@ -134,74 +133,6 @@
     <t>date</t>
   </si>
   <si>
-    <r>
-      <t>ERS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFCCCCCC"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>Patient</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFCCCCCC"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>Transport</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFCCCCCC"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t>Service</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FFCCCCCC"/>
-        <rFont val="Consolas"/>
-        <family val="3"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-  </si>
-  <si>
     <t>note</t>
   </si>
   <si>
@@ -226,15 +157,6 @@
       </rPr>
       <t>Note</t>
     </r>
-  </si>
-  <si>
-    <t>chargeCategory</t>
-  </si>
-  <si>
-    <t>ValidData</t>
-  </si>
-  <si>
-    <t>testcase</t>
   </si>
 </sst>
 </file>
@@ -620,107 +542,47 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.6640625" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" customWidth="1"/>
-    <col min="3" max="3" width="35.5546875" customWidth="1"/>
+    <col min="2" max="2" width="34.6640625" customWidth="1"/>
+    <col min="3" max="3" width="11.88671875" customWidth="1"/>
     <col min="4" max="4" width="14.88671875" customWidth="1"/>
     <col min="5" max="5" width="31" customWidth="1"/>
     <col min="6" max="6" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>9</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="3">
+      <c r="A2" s="3">
         <v>1185</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="4">
+      <c r="C2" s="4">
         <v>46159</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58089021-8731-4835-8BC8-833E2A1D40E3}">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="34.5546875" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" customWidth="1"/>
-    <col min="4" max="4" width="30.21875" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
-        <v>1185</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="4">
-        <v>46159</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>